<commit_message>
Pare the archive labels back to their first lines
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/ninefold-copy-sheet.xlsx
+++ b/ninefold-copy-sheet.xlsx
@@ -8958,12 +8958,12 @@
       </c>
       <c r="E250" s="11" t="inlineStr">
         <is>
-          <t>THE ARCHIVE REMEMBERS&lt;br&gt;WHAT THE BODY COULD NOT SAY</t>
+          <t>&amp;ldquo;sponge,&lt;br&gt;you shall dry again&amp;rdquo;</t>
         </is>
       </c>
       <c r="F250" s="9" t="n"/>
       <c r="G250" s="10" t="n">
-        <v>52</v>
+        <v>44</v>
       </c>
       <c r="H250" s="11" t="inlineStr"/>
     </row>
@@ -8988,12 +8988,12 @@
       </c>
       <c r="E251" s="11" t="inlineStr">
         <is>
-          <t>3 FRAGMENTS HAVE RETURNED&lt;br&gt;THE REST ARE WAITING IN THE DARK</t>
+          <t>3 FRAGMENTS HAVE RETURNED</t>
         </is>
       </c>
       <c r="F251" s="9" t="n"/>
       <c r="G251" s="10" t="n">
-        <v>61</v>
+        <v>25</v>
       </c>
       <c r="H251" s="11" t="inlineStr"/>
     </row>
@@ -9052,12 +9052,12 @@
       </c>
       <c r="E253" s="11" t="inlineStr">
         <is>
-          <t>THE FIRST FRAGMENT SURFACES&lt;br&gt;WHAT WAS BURIED KEEPS SPEAKING</t>
+          <t>FRAGMENT 01</t>
         </is>
       </c>
       <c r="F253" s="9" t="n"/>
       <c r="G253" s="10" t="n">
-        <v>61</v>
+        <v>11</v>
       </c>
       <c r="H253" s="11" t="inlineStr"/>
     </row>
@@ -9218,16 +9218,16 @@
       </c>
       <c r="E258" s="11" t="inlineStr">
         <is>
-          <t>ONE FRAGMENT HAS RETURNED&lt;br&gt;THE REST ARE WAITING IN THE DARK</t>
+          <t>ONE FRAGMENT HAS RETURNED</t>
         </is>
       </c>
       <c r="F258" s="9" t="n"/>
       <c r="G258" s="10" t="n">
-        <v>61</v>
+        <v>25</v>
       </c>
       <c r="H258" s="11" t="inlineStr">
         <is>
-          <t xml:space="preserve">if (unlocked === 1) return 'ONE FRAGMENT HAS RETURNED&lt;br&gt;THE REST ARE </t>
+          <t>if (unlocked === 1) return 'ONE FRAGMENT HAS RETURNED';</t>
         </is>
       </c>
     </row>
@@ -9252,16 +9252,16 @@
       </c>
       <c r="E259" s="11" t="inlineStr">
         <is>
-          <t>${unlocked} FRAGMENTS HAVE RETURNED&lt;br&gt;THE REST ARE WAITING IN THE DARK</t>
+          <t>${unlocked} FRAGMENTS HAVE RETURNED</t>
         </is>
       </c>
       <c r="F259" s="9" t="n"/>
       <c r="G259" s="10" t="n">
-        <v>71</v>
+        <v>35</v>
       </c>
       <c r="H259" s="11" t="inlineStr">
         <is>
-          <t>return `${unlocked} FRAGMENTS HAVE RETURNED&lt;br&gt;THE REST ARE WAITING IN</t>
+          <t>return `${unlocked} FRAGMENTS HAVE RETURNED`;</t>
         </is>
       </c>
     </row>
@@ -9422,16 +9422,16 @@
       </c>
       <c r="E264" s="11" t="inlineStr">
         <is>
-          <t>FRAGMENT ${ordinal} SURFACES&lt;br&gt;WHAT WAS BURIED KEEPS SPEAKING</t>
+          <t>FRAGMENT ${ordinal}</t>
         </is>
       </c>
       <c r="F264" s="9" t="n"/>
       <c r="G264" s="10" t="n">
-        <v>62</v>
+        <v>19</v>
       </c>
       <c r="H264" s="11" t="inlineStr">
         <is>
-          <t>$('#archive-reader-label').innerHTML = `FRAGMENT ${ordinal} SURFACES&lt;b</t>
+          <t>$('#archive-reader-label').innerHTML = `FRAGMENT ${ordinal}`;</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Tighten the fragment count line
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/ninefold-copy-sheet.xlsx
+++ b/ninefold-copy-sheet.xlsx
@@ -8988,12 +8988,12 @@
       </c>
       <c r="E251" s="11" t="inlineStr">
         <is>
-          <t>3 FRAGMENTS HAVE RETURNED</t>
+          <t>3 FRAGMENTS RETURNED</t>
         </is>
       </c>
       <c r="F251" s="9" t="n"/>
       <c r="G251" s="10" t="n">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="H251" s="11" t="inlineStr"/>
     </row>
@@ -9252,16 +9252,16 @@
       </c>
       <c r="E259" s="11" t="inlineStr">
         <is>
-          <t>${unlocked} FRAGMENTS HAVE RETURNED</t>
+          <t>${unlocked} FRAGMENTS RETURNED</t>
         </is>
       </c>
       <c r="F259" s="9" t="n"/>
       <c r="G259" s="10" t="n">
-        <v>35</v>
+        <v>30</v>
       </c>
       <c r="H259" s="11" t="inlineStr">
         <is>
-          <t>return `${unlocked} FRAGMENTS HAVE RETURNED`;</t>
+          <t>return `${unlocked} FRAGMENTS RETURNED`;</t>
         </is>
       </c>
     </row>

</xml_diff>